<commit_message>
Updated ouput variables to support testing at dataset level without split datasets.
</commit_message>
<xml_diff>
--- a/rules/CORE-000365/negative/01/data/unit-test-coreid-CG0077-negative 1.xlsx
+++ b/rules/CORE-000365/negative/01/data/unit-test-coreid-CG0077-negative 1.xlsx
@@ -523,7 +523,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F3"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -546,68 +546,48 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="str">
+      <c r="B2" s="2" t="str">
         <v>mh.xpt</v>
       </c>
-      <c r="C2" s="4" t="str">
+      <c r="C2" s="2" t="str">
         <v>Record</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="2">
         <v>5</v>
       </c>
-      <c r="E2" s="4" t="str">
+      <c r="E2" s="2" t="str">
+        <v>USUBJID</v>
+      </c>
+      <c r="F2" s="2" t="str">
+        <v>CDISC010</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="str">
+        <v>mh.xpt</v>
+      </c>
+      <c r="C3" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D3" s="4">
+        <v>5</v>
+      </c>
+      <c r="E3" s="4" t="str">
         <v>MHCAT</v>
       </c>
-      <c r="F2" s="4" t="str">
-        <v>GENERAL</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="str">
-        <v>mh.xpt</v>
-      </c>
-      <c r="C3" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D3" s="2">
-        <v>6</v>
-      </c>
-      <c r="E3" s="2" t="str">
-        <v>MHCAT</v>
-      </c>
-      <c r="F3" s="2" t="str">
-        <v>GENERAL</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="str">
-        <v>mh.xpt</v>
-      </c>
-      <c r="C4" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D4" s="2">
-        <v>7</v>
-      </c>
-      <c r="E4" s="2" t="str">
-        <v>MHCAT</v>
-      </c>
-      <c r="F4" s="2" t="str">
+      <c r="F3" s="4" t="str">
         <v>GENERAL</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -649,10 +629,10 @@
       <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="6" t="str">
+      <c r="B2" s="5" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="6" t="str">
+      <c r="C2" s="5" t="str">
         <v>Unique Subject Identifier</v>
       </c>
       <c r="D2" s="6" t="str">
@@ -739,13 +719,13 @@
       <c r="B5" s="4" t="str">
         <v>MH</v>
       </c>
-      <c r="C5" s="4" t="str">
+      <c r="C5" s="7" t="str">
         <v>CDISC010</v>
       </c>
       <c r="D5" s="4">
         <v>1</v>
       </c>
-      <c r="E5" s="7" t="str">
+      <c r="E5" s="8" t="str">
         <v>GENERAL</v>
       </c>
       <c r="F5" s="4" t="str">
@@ -765,7 +745,7 @@
       <c r="D6" s="4">
         <v>1</v>
       </c>
-      <c r="E6" s="8" t="str">
+      <c r="E6" s="4" t="str">
         <v>GENERAL</v>
       </c>
       <c r="F6" s="4" t="str">
@@ -785,7 +765,7 @@
       <c r="D7" s="4">
         <v>1</v>
       </c>
-      <c r="E7" s="8" t="str">
+      <c r="E7" s="4" t="str">
         <v>GENERAL</v>
       </c>
       <c r="F7" s="4" t="str">

</xml_diff>

<commit_message>
Removed USUBJID from the output variables as requested.
</commit_message>
<xml_diff>
--- a/rules/CORE-000365/negative/01/data/unit-test-coreid-CG0077-negative 1.xlsx
+++ b/rules/CORE-000365/negative/01/data/unit-test-coreid-CG0077-negative 1.xlsx
@@ -36,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -62,18 +62,9 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="4">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -87,18 +78,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFCC"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -128,7 +107,7 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -136,8 +115,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -523,7 +500,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -546,48 +523,28 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>mh.xpt</v>
       </c>
-      <c r="C2" s="2" t="str">
+      <c r="C2" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="4">
         <v>5</v>
       </c>
-      <c r="E2" s="2" t="str">
-        <v>USUBJID</v>
-      </c>
-      <c r="F2" s="2" t="str">
-        <v>CDISC010</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="str">
-        <v>mh.xpt</v>
-      </c>
-      <c r="C3" s="4" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D3" s="4">
-        <v>5</v>
-      </c>
-      <c r="E3" s="4" t="str">
+      <c r="E2" s="4" t="str">
         <v>MHCAT</v>
       </c>
-      <c r="F3" s="4" t="str">
+      <c r="F2" s="4" t="str">
         <v>GENERAL</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -635,80 +592,80 @@
       <c r="C2" s="5" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="6" t="str">
+      <c r="D2" s="5" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="E2" s="6" t="str">
+      <c r="E2" s="5" t="str">
         <v>Category for Medical History</v>
       </c>
-      <c r="F2" s="6" t="str">
+      <c r="F2" s="5" t="str">
         <v>Reported Term for the Medical History</v>
       </c>
-      <c r="G2" s="6" t="str">
+      <c r="G2" s="5" t="str">
         <v>Medical History Event Date Type</v>
       </c>
-      <c r="H2" s="6" t="str">
+      <c r="H2" s="5" t="str">
         <v>Start Date/Time of Medical History Event</v>
       </c>
-      <c r="I2" s="6" t="str">
+      <c r="I2" s="5" t="str">
         <v>Study Day of Start of Observation</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="str">
+      <c r="A3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="B3" s="6" t="str">
+      <c r="B3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="C3" s="6" t="str">
+      <c r="C3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="D3" s="6" t="str">
+      <c r="D3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="E3" s="6" t="str">
+      <c r="E3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="F3" s="6" t="str">
+      <c r="F3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="G3" s="6" t="str">
+      <c r="G3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="H3" s="6" t="str">
+      <c r="H3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="I3" s="6" t="str">
+      <c r="I3" s="5" t="str">
         <v>Num</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6">
+      <c r="A4" s="5">
         <v>12</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="5">
         <v>2</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="5">
         <v>8</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="5">
         <v>8</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="5">
         <v>50</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="5">
         <v>19</v>
       </c>
-      <c r="G4" s="6">
+      <c r="G4" s="5">
         <v>13</v>
       </c>
-      <c r="H4" s="6">
+      <c r="H4" s="5">
         <v>10</v>
       </c>
-      <c r="I4" s="6">
+      <c r="I4" s="5">
         <v>8</v>
       </c>
     </row>
@@ -719,13 +676,13 @@
       <c r="B5" s="4" t="str">
         <v>MH</v>
       </c>
-      <c r="C5" s="7" t="str">
+      <c r="C5" s="4" t="str">
         <v>CDISC010</v>
       </c>
       <c r="D5" s="4">
         <v>1</v>
       </c>
-      <c r="E5" s="8" t="str">
+      <c r="E5" s="6" t="str">
         <v>GENERAL</v>
       </c>
       <c r="F5" s="4" t="str">

</xml_diff>